<commit_message>
Update roles spreadsheet with adjacent titles (strategy ops, director ops, VP ops, COO)
</commit_message>
<xml_diff>
--- a/Chief_of_Staff_Roles_Mar2026.xlsx
+++ b/Chief_of_Staff_Roles_Mar2026.xlsx
@@ -7,8 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NYC Metro" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Remote (US, non-CA)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chief of Staff (NYC)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Strategy &amp; Ops (NYC)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Director of Ops (NYC)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="VP Operations (NYC)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="COO (NYC)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Remote (non-CA)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +40,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +51,36 @@
       <patternFill patternType="solid">
         <fgColor rgb="002B5797"/>
         <bgColor rgb="002B5797"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A7A3A"/>
+        <bgColor rgb="001A7A3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B4513"/>
+        <bgColor rgb="008B4513"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006B2D8B"/>
+        <bgColor rgb="006B2D8B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0392B"/>
+        <bgColor rgb="00C0392B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002C3E50"/>
+        <bgColor rgb="002C3E50"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,13 +102,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,9 +492,9 @@
   <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1134,38 +1183,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Posted</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Apply Link</t>
         </is>
@@ -1174,22 +1223,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Optum</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff - Remote</t>
+          <t>Strategy and Operations Lead</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>3 hours ago</t>
+          <t>4 days ago</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -1201,22 +1250,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Perpay Inc.</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Strategy and Operations Senior Associate</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Philadelphia, PA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>8 hours ago</t>
+          <t>1 week ago</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -1228,22 +1277,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Jobgether</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Strategy and Operations Lead, Americas PGTM</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>4 days ago</t>
+          <t>5 days ago</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -1255,22 +1304,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Jack &amp; Jill / Dealflowagent</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff (Founding Operator) — $100-140k + equity</t>
+          <t>Strategy and Operations Senior Associate, GTM</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>5 days ago</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1282,22 +1331,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Coinbase</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff to the COO</t>
+          <t>Strategy and Operations Senior Associate, gTech</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>1 day ago</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -1309,22 +1358,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Serve Freight</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff - Executive Ops</t>
+          <t>Strategy and Operations Senior Analyst</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1 week ago</t>
+          <t>2 weeks ago</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1336,17 +1385,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>LEE</t>
+          <t>Twitch</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff to the President (Temp)</t>
+          <t>Senior Manager, Strategy and Operations</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1363,17 +1412,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Fannie Mae</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>VP, Chief of Staff for Head of Marketing</t>
+          <t>Partner Strategy &amp; Operations Manager</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1390,17 +1439,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Zelis</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Director, Chief of Staff, Marketing</t>
+          <t>Strategic Planning and Operations Manager, Business Marketing</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Remote (FL/NJ)</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1417,22 +1466,828 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Revecore</t>
+          <t>Fanatics</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Chief of Staff</t>
+          <t>Director, Strategy and Business Operations</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1 month ago</t>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Senior Manager, Business Operations &amp; Strategy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Suno</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Senior Manager, Business Operations &amp; Strategy</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Savant Bio</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Strategy and Operations Lead</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Rockstar Games</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Strategy Operations Associate</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Manhattan, NY</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>16 hours ago</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SentiLink</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Business Operations Associate</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>3 days ago</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Flex</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Director, Strategy &amp; Operations (Housing)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Whatnot</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Director, Strategy &amp; Operations - Service Delivery</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Greylock Partners</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Strategy and Business Operations Lead (Seed Stage)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>NYC Metro</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>M7 Health</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Strategy &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Plaid</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Sales Operations Associate, GTM Strategy &amp; Ops</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Director, Sales Strategy &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Operations Manager, Uber Eats</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Senior Strategic Operations Manager, Delivery</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Hopper</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Senior Strategy &amp; Operations Manager - HTS Media (100% Remote)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Garage</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>People Strategy &amp; Operations Lead</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>1 day ago</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>MrBeast</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Associate, Strategic Finance</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>A24</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Financial Analyst, Corporate Finance &amp; Strategy</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>4 days ago</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Apply Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Trueline</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Director of Operations</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Colts Neck, NJ</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1 day ago</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SoulCycle</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Senior Director, Operations, Facilities &amp; Bike Ops</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>5 days ago</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sol de Janeiro</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Executive Director, Fulfillment Operations - Americas</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>NYC Metro</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GiveDirectly</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Senior Global Director of Country Operations (Remote)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Neura Health</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Fractional COO / VP of Operations</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Wild</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Associate Operations Director</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Convene</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Director of Operations - NeueHouse Madison Square</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Nomad</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Director of Operations</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>3 weeks ago</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Recora</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Manager, Executive Operations</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>3 weeks ago</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Head of Retail Operations</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>5 days ago</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1456,4 +2311,882 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Apply Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Razorfish</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>VP, Media Operations</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>5 hours ago</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Dow Jones</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>VP, Strategy &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2 days ago</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Gartner</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>VP, Product Strategy &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Stamford, CT</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>3 days ago</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Brooklinen</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SVP, Operations</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>3 weeks ago</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>dentsu</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EVP, Growth Operations</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Broadridge</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>VP, Strategy and Business Development (Hybrid)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Newark, NJ</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>IPC Systems</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>SVP, Strategic Planning &amp; Analysis</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Cohen &amp; Steers</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>VP, AI Strategy &amp; Enablement</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LevelUP HCS</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>VP Corporate Strategy</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>4 days ago</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Veho</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Sr. VP of Supply Chain</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Sesame Workshop</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>VP, Business Development &amp; Growth Strategy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2 weeks ago</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Apply Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Risk COO (Risk Management)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Neura Health</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Fractional COO / VP of Operations</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>JPMorganChase</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy VP, Global Technology Transformation</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>5 days ago</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Apply Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff - Remote</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>3 hours ago</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Perpay Inc.</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>8 hours ago</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>4 days ago</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Jack &amp; Jill / Dealflowagent</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff (Founding Operator) — $100-140k + equity</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Coinbase</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the COO</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Serve Freight</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff - Executive Ops</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>LEE</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff to the President (Temp)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Fannie Mae</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>VP, Chief of Staff for Head of Marketing</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Washington, DC</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Zelis</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Director, Chief of Staff, Marketing</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Remote (FL/NJ)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Revecore</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Chief of Staff</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1 month ago</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>GiveDirectly</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Senior Global Director of Country Operations (Remote)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Hopper</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Senior Strategy &amp; Operations Manager - HTS Media (100% Remote)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Remote</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>1 week ago</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Apply →</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>